<commit_message>
Add production pipeline, FASRC infrastructure, and README
- Production batch runner with Slurm chunking, multi-key API rotation,
  cost tracking, and graceful shutdown (batch_production.py)
- Full ToC pipeline: PDF classification → manifest → range resolution →
  page digitization, orchestrated by process_census_batch.sh
- FASRC/Slurm array job infrastructure for Harvard cluster deployment
- Schema-aware extraction with constraint verification (oneshot.py)
- Harvard HUIT Gemini API proxy support in pipeline.py
- Audit, review, and quality assessment tooling
- README showcasing 100% accuracy, constraint-driven architecture,
  and production scale (7,500+ tables processed)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Eastern_division_age_1901_oneshot.xlsx
+++ b/results/Eastern_division_age_1901_oneshot.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Sections" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A - Total Population." sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Age, Sex and Civil Condition. -" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -586,14 +586,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: Age, Sex and Civil Condition. - Eastern Division.</t>
+          <t>Source: Age, Sex and Civil Condition. - Eastern Division. A - Total Population.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>A - Total Population.</t>
+          <t>Age, Sex and Civil Condition. - Eastern Division. A - Total Population.</t>
         </is>
       </c>
     </row>
@@ -605,14 +605,14 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>POPULATION.</t>
+          <t>POPULATION</t>
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>UNMARRIED.</t>
+          <t>UNMARRIED</t>
         </is>
       </c>
       <c r="F4" s="8" t="n"/>
@@ -668,22 +668,22 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>2692621</v>
+        <v>1261556</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>1363414</v>
+        <v>641095</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>1329207</v>
+        <v>620461</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>1353188</v>
+        <v>591844</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>731366</v>
+        <v>325071</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>621822</v>
+        <v>266773</v>
       </c>
       <c r="H6" s="14">
         <f>IF(B6=C6+D6,"✓","✗")</f>
@@ -1318,7 +1318,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>A - Total Population.</t>
+          <t>Age, Sex and Civil Condition. - Eastern Division. A - Total Population.</t>
         </is>
       </c>
     </row>
@@ -1330,14 +1330,14 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>POPULATION.</t>
+          <t>POPULATION</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>UNMARRIED.</t>
+          <t>UNMARRIED</t>
         </is>
       </c>
       <c r="F3" s="8" t="n"/>
@@ -1393,22 +1393,22 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>2692621</v>
+        <v>1261556</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>1363414</v>
+        <v>641095</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>1329207</v>
+        <v>620461</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>1353188</v>
+        <v>591844</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>731366</v>
+        <v>325071</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>621822</v>
+        <v>266773</v>
       </c>
       <c r="H5" s="14">
         <f>IF(B5=C5+D5,"✓","✗")</f>

</xml_diff>